<commit_message>
inputs: one Contents standard, units in numeric order
Every per-book input spreadsheet now uses the site's Contents format
(Section type | Title | Page), converted from the raw Odoo scheme-of-work
exports: the unit name repeats on every row there, the subunit sits in a
later column, and one export column carried the id, so units were read as
subunits and y02/y04 computing began at Unit 5 then jumped to Unit 1.

Units are now emitted in numeric order, each immediately followed by its
own subunits in order; term revision/assessment rows become Section rows.
Raw originals are preserved under public/inputs-raw/.
</commit_message>
<xml_diff>
--- a/public/inputs/y01-art-and-design - input.xlsx
+++ b/public/inputs/y01-art-and-design - input.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001D7A3D"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,24 +415,19 @@
   </sheetPr>
   <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Section type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Page</t>
         </is>
@@ -459,9 +444,7 @@
           <t>Unit 1 · The Mark Room</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>8</v>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -474,8 +457,10 @@
           <t>1.1 Marks and lines</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>11</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -489,8 +474,10 @@
           <t>1.2 Drawing tools</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>16</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -504,8 +491,10 @@
           <t>1.3 Looking and drawing</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>19</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -519,8 +508,10 @@
           <t>1.4 My own project</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>22</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -534,9 +525,7 @@
           <t>Unit 2 · The Thread Room</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>25</v>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -549,8 +538,10 @@
           <t>2.1 Weaving</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>29</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -564,8 +555,10 @@
           <t>2.2 Stitch and lace</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>31</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -579,8 +572,10 @@
           <t>2.3 My textile</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>35</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -594,8 +589,10 @@
           <t>2.4 Colour and texture</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>37</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -609,9 +606,7 @@
           <t>Unit 3 · The Clay Room</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>42</v>
-      </c>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -624,8 +619,10 @@
           <t>3.1 Solid forms</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>45</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -639,8 +636,10 @@
           <t>3.2 Materials</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>48</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -654,8 +653,10 @@
           <t>3.3 Texture</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>50</v>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -669,8 +670,10 @@
           <t>3.4 My sculpture</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>52</v>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -684,9 +687,7 @@
           <t>Unit 4 · The Paint Room</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>57</v>
-      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -699,8 +700,10 @@
           <t>4.1 Brushes and tools</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>60</v>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -714,8 +717,10 @@
           <t>4.2 Mixing colour</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>62</v>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -729,8 +734,10 @@
           <t>4.3 Small and big</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>66</v>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -744,8 +751,10 @@
           <t>4.4 My painting</t>
         </is>
       </c>
-      <c r="C21" t="n">
-        <v>67</v>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -759,8 +768,10 @@
           <t>Our studio show</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>72</v>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -774,8 +785,10 @@
           <t>My portfolio</t>
         </is>
       </c>
-      <c r="C23" t="n">
-        <v>74</v>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -789,8 +802,10 @@
           <t>Art all through the year</t>
         </is>
       </c>
-      <c r="C24" t="n">
-        <v>76</v>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -804,8 +819,10 @@
           <t>My word book</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>78</v>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -819,8 +836,10 @@
           <t>Where we found out</t>
         </is>
       </c>
-      <c r="C26" t="n">
-        <v>86</v>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>